<commit_message>
Added Two Tests in Add Patient feature
</commit_message>
<xml_diff>
--- a/Python-Automation-SmartHospital/data_files/AddPatientdetails.xlsx
+++ b/Python-Automation-SmartHospital/data_files/AddPatientdetails.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5995a90617affbed/Desktop/smartHospitalPython/Python-Automation-SmartHospital/data_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{8782617A-6E87-4823-8BE1-DFB8C58792FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{402EFA0B-AD6D-47FF-A6C4-47F3D048C97A}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="8_{8782617A-6E87-4823-8BE1-DFB8C58792FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{139CC003-47C9-4ACF-B696-5E10CB2544C3}"/>
   <bookViews>
-    <workbookView xWindow="4188" yWindow="3360" windowWidth="17832" windowHeight="8880" xr2:uid="{8600487F-118E-4B1E-A562-436AAA0E569F}"/>
+    <workbookView xWindow="4188" yWindow="3360" windowWidth="17832" windowHeight="8880" activeTab="2" xr2:uid="{8600487F-118E-4B1E-A562-436AAA0E569F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
   <si>
     <t>Name</t>
   </si>
@@ -76,13 +78,76 @@
   </si>
   <si>
     <t>Bangalore</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>guardian</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>dob</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>blood_group</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>142879f</t>
+  </si>
+  <si>
+    <t>valid@mail.com</t>
+  </si>
+  <si>
+    <t>B+</t>
+  </si>
+  <si>
+    <t>Chennai</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>jannx@546@gamil.com</t>
+  </si>
+  <si>
+    <t>A+</t>
+  </si>
+  <si>
+    <t>Mumbai</t>
+  </si>
+  <si>
+    <t>Ram</t>
+  </si>
+  <si>
+    <t>Henry</t>
+  </si>
+  <si>
+    <t>Pooja</t>
+  </si>
+  <si>
+    <t>vinai</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy/mm/dd\ h:mm:ss"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,16 +171,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -123,12 +207,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -141,6 +240,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -158,10 +266,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -522,4 +626,128 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D9DB56F-5E5F-4A73-BA9B-CF352718915A}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="7">
+        <v>33003</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31596C97-0E33-410A-A3CA-FB659BC019DB}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="7">
+        <v>34165</v>
+      </c>
+      <c r="E2" s="6">
+        <v>9876543213</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>